<commit_message>
Modificado margenes de actas
</commit_message>
<xml_diff>
--- a/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
+++ b/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyecto\ControlActivosTI\ControlActivosTI\templates\actas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A692F23-6B3A-4B62-B2D9-9C8BFF29B16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B121A06-7E1F-4726-BE66-68D2EE067B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14290" yWindow="-1820" windowWidth="19420" windowHeight="10300" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13740" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1029,6 +1029,309 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1067,309 +1370,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1787,42 +1787,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="25" t="e" vm="1">
+      <c r="B1" s="89" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="31" t="s">
+      <c r="C1" s="90"/>
+      <c r="D1" s="93" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34" t="s">
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="36" t="s">
+      <c r="I1" s="98" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="27"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="38" t="s">
+      <c r="B2" s="91"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="37"/>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="99"/>
     </row>
     <row r="3" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="27"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="118"/>
-      <c r="F3" s="118"/>
-      <c r="G3" s="42"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="105"/>
       <c r="H3" s="2" t="s">
         <v>2</v>
       </c>
@@ -1831,120 +1831,120 @@
       </c>
     </row>
     <row r="4" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="27"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="118"/>
-      <c r="F4" s="118"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="46" t="s">
+      <c r="B4" s="91"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="105"/>
+      <c r="H4" s="109" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="48">
+      <c r="I4" s="111">
         <v>46097</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="29"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="44"/>
-      <c r="F5" s="44"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="49"/>
+      <c r="B5" s="92"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="110"/>
+      <c r="I5" s="112"/>
     </row>
     <row r="6" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="51"/>
-      <c r="D6" s="52"/>
-      <c r="E6" s="73"/>
-      <c r="F6" s="74"/>
-      <c r="G6" s="74"/>
-      <c r="H6" s="74"/>
-      <c r="I6" s="75"/>
+      <c r="C6" s="69"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
+      <c r="I6" s="86"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="64" t="s">
+      <c r="B7" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="C7" s="65"/>
-      <c r="D7" s="65"/>
-      <c r="E7" s="65"/>
-      <c r="F7" s="65"/>
-      <c r="G7" s="65"/>
-      <c r="H7" s="65"/>
-      <c r="I7" s="66"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="25"/>
+      <c r="G7" s="25"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="26"/>
     </row>
     <row r="8" spans="2:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="53"/>
-      <c r="C8" s="119"/>
-      <c r="D8" s="119"/>
-      <c r="E8" s="119"/>
-      <c r="F8" s="119"/>
-      <c r="G8" s="119"/>
-      <c r="H8" s="119"/>
-      <c r="I8" s="54"/>
+      <c r="B8" s="21"/>
+      <c r="C8" s="22"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
+      <c r="I8" s="23"/>
     </row>
     <row r="9" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="53"/>
-      <c r="C9" s="119"/>
-      <c r="D9" s="119"/>
-      <c r="E9" s="119"/>
-      <c r="F9" s="119"/>
-      <c r="G9" s="119"/>
-      <c r="H9" s="119"/>
-      <c r="I9" s="54"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="124" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="18" t="s">
+      <c r="C10" s="119"/>
+      <c r="D10" s="119"/>
+      <c r="E10" s="125"/>
+      <c r="F10" s="125"/>
+      <c r="G10" s="125"/>
+      <c r="H10" s="119" t="s">
         <v>14</v>
       </c>
-      <c r="I10" s="19"/>
+      <c r="I10" s="120"/>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="78" t="s">
+      <c r="B11" s="87" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="79"/>
-      <c r="D11" s="79"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="19"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="116"/>
+      <c r="F11" s="117"/>
+      <c r="G11" s="118"/>
+      <c r="H11" s="119"/>
+      <c r="I11" s="120"/>
     </row>
     <row r="12" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="20" t="s">
+      <c r="B12" s="121" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="22"/>
+      <c r="C12" s="122"/>
+      <c r="D12" s="122"/>
+      <c r="E12" s="122"/>
+      <c r="F12" s="122"/>
+      <c r="G12" s="122"/>
+      <c r="H12" s="122"/>
+      <c r="I12" s="123"/>
     </row>
     <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="67" t="s">
+      <c r="B13" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="68"/>
-      <c r="D13" s="68" t="s">
+      <c r="C13" s="79"/>
+      <c r="D13" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="68"/>
+      <c r="E13" s="79"/>
       <c r="F13" s="10" t="s">
         <v>37</v>
       </c>
@@ -1959,626 +1959,628 @@
       </c>
     </row>
     <row r="14" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="69"/>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="61"/>
+      <c r="B14" s="80"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="9"/>
     </row>
     <row r="15" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="13"/>
+      <c r="B15" s="113"/>
+      <c r="C15" s="114"/>
+      <c r="D15" s="115"/>
+      <c r="E15" s="114"/>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
     </row>
     <row r="16" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="76"/>
-      <c r="C16" s="77"/>
-      <c r="D16" s="77"/>
-      <c r="E16" s="77"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="2:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="62"/>
-      <c r="C17" s="63"/>
-      <c r="D17" s="63"/>
-      <c r="E17" s="63"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="7"/>
     </row>
     <row r="18" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="83" t="s">
+      <c r="B18" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="84"/>
-      <c r="D18" s="84"/>
-      <c r="E18" s="84"/>
-      <c r="F18" s="84"/>
-      <c r="G18" s="84"/>
-      <c r="H18" s="84"/>
-      <c r="I18" s="85"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="32"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="97" t="s">
+      <c r="B19" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="98"/>
-      <c r="D19" s="98"/>
-      <c r="E19" s="98"/>
-      <c r="F19" s="98" t="s">
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="G19" s="98"/>
-      <c r="H19" s="98" t="s">
+      <c r="G19" s="34"/>
+      <c r="H19" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="I19" s="99"/>
+      <c r="I19" s="35"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="76" t="s">
+      <c r="B20" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="77"/>
-      <c r="D20" s="77"/>
-      <c r="E20" s="77"/>
-      <c r="F20" s="106"/>
-      <c r="G20" s="106"/>
-      <c r="H20" s="100" t="s">
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="38" t="s">
         <v>41</v>
       </c>
-      <c r="I20" s="101"/>
+      <c r="I20" s="39"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="76" t="s">
+      <c r="B21" s="44" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="77"/>
-      <c r="D21" s="77"/>
-      <c r="E21" s="77"/>
-      <c r="F21" s="106"/>
-      <c r="G21" s="106"/>
-      <c r="H21" s="102"/>
-      <c r="I21" s="101"/>
+      <c r="C21" s="45"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="39"/>
     </row>
     <row r="22" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="62" t="s">
+      <c r="B22" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="63"/>
-      <c r="D22" s="63"/>
-      <c r="E22" s="63"/>
-      <c r="F22" s="105"/>
-      <c r="G22" s="105"/>
-      <c r="H22" s="103"/>
-      <c r="I22" s="104"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="42"/>
     </row>
     <row r="23" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="70" t="s">
+      <c r="B23" s="81" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="71"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="71"/>
-      <c r="F23" s="71"/>
-      <c r="G23" s="71"/>
-      <c r="H23" s="71"/>
-      <c r="I23" s="72"/>
+      <c r="C23" s="82"/>
+      <c r="D23" s="82"/>
+      <c r="E23" s="82"/>
+      <c r="F23" s="82"/>
+      <c r="G23" s="82"/>
+      <c r="H23" s="82"/>
+      <c r="I23" s="83"/>
     </row>
     <row r="24" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="53" t="s">
+      <c r="B24" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="119"/>
-      <c r="D24" s="119"/>
-      <c r="E24" s="119"/>
-      <c r="F24" s="119"/>
-      <c r="G24" s="119"/>
-      <c r="H24" s="119"/>
-      <c r="I24" s="54"/>
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="23"/>
     </row>
     <row r="25" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="53"/>
-      <c r="C25" s="119"/>
-      <c r="D25" s="119"/>
-      <c r="E25" s="119"/>
-      <c r="F25" s="119"/>
-      <c r="G25" s="119"/>
-      <c r="H25" s="119"/>
-      <c r="I25" s="54"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="23"/>
     </row>
     <row r="26" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="53" t="s">
+      <c r="B26" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="119"/>
-      <c r="D26" s="119"/>
-      <c r="E26" s="119"/>
-      <c r="F26" s="119"/>
-      <c r="G26" s="119"/>
-      <c r="H26" s="119"/>
-      <c r="I26" s="54"/>
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="23"/>
     </row>
     <row r="27" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="53" t="s">
+      <c r="B27" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="119"/>
-      <c r="D27" s="119"/>
-      <c r="E27" s="119"/>
-      <c r="F27" s="119"/>
-      <c r="G27" s="119"/>
-      <c r="H27" s="119"/>
-      <c r="I27" s="54"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="23"/>
     </row>
     <row r="28" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="53" t="s">
+      <c r="B28" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="119"/>
-      <c r="D28" s="119"/>
-      <c r="E28" s="119"/>
-      <c r="F28" s="119"/>
-      <c r="G28" s="119"/>
-      <c r="H28" s="119"/>
-      <c r="I28" s="54"/>
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="23"/>
     </row>
     <row r="29" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="53" t="s">
+      <c r="B29" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="C29" s="119"/>
-      <c r="D29" s="119"/>
-      <c r="E29" s="119"/>
-      <c r="F29" s="119"/>
-      <c r="G29" s="119"/>
-      <c r="H29" s="119"/>
-      <c r="I29" s="54"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="23"/>
     </row>
     <row r="30" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="53" t="s">
+      <c r="B30" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="119"/>
-      <c r="D30" s="119"/>
-      <c r="E30" s="119"/>
-      <c r="F30" s="119"/>
-      <c r="G30" s="119"/>
-      <c r="H30" s="119"/>
-      <c r="I30" s="54"/>
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="I30" s="23"/>
     </row>
     <row r="31" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="53" t="s">
+      <c r="B31" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="119"/>
-      <c r="D31" s="119"/>
-      <c r="E31" s="119"/>
-      <c r="F31" s="119"/>
-      <c r="G31" s="119"/>
-      <c r="H31" s="119"/>
-      <c r="I31" s="54"/>
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="I31" s="23"/>
     </row>
     <row r="32" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="53" t="s">
+      <c r="B32" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C32" s="119"/>
-      <c r="D32" s="119"/>
-      <c r="E32" s="119"/>
-      <c r="F32" s="119"/>
-      <c r="G32" s="119"/>
-      <c r="H32" s="119"/>
-      <c r="I32" s="54"/>
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="23"/>
     </row>
     <row r="33" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="53" t="s">
+      <c r="B33" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="119"/>
-      <c r="D33" s="119"/>
-      <c r="E33" s="119"/>
-      <c r="F33" s="119"/>
-      <c r="G33" s="119"/>
-      <c r="H33" s="119"/>
-      <c r="I33" s="54"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="23"/>
     </row>
     <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="53" t="s">
+      <c r="B34" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C34" s="119"/>
-      <c r="D34" s="119"/>
-      <c r="E34" s="119"/>
-      <c r="F34" s="119"/>
-      <c r="G34" s="119"/>
-      <c r="H34" s="119"/>
-      <c r="I34" s="54"/>
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="23"/>
     </row>
     <row r="35" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="53"/>
-      <c r="C35" s="119"/>
-      <c r="D35" s="119"/>
-      <c r="E35" s="119"/>
-      <c r="F35" s="119"/>
-      <c r="G35" s="119"/>
-      <c r="H35" s="119"/>
-      <c r="I35" s="54"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="22"/>
+      <c r="D35" s="22"/>
+      <c r="E35" s="22"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="I35" s="23"/>
     </row>
     <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="53" t="s">
+      <c r="B36" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="C36" s="119"/>
-      <c r="D36" s="119"/>
-      <c r="E36" s="119"/>
-      <c r="F36" s="119"/>
-      <c r="G36" s="119"/>
-      <c r="H36" s="119"/>
-      <c r="I36" s="54"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="22"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="I36" s="23"/>
     </row>
     <row r="37" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="55"/>
-      <c r="C37" s="56"/>
-      <c r="D37" s="56"/>
-      <c r="E37" s="56"/>
-      <c r="F37" s="56"/>
-      <c r="G37" s="56"/>
-      <c r="H37" s="56"/>
-      <c r="I37" s="57"/>
+      <c r="B37" s="71"/>
+      <c r="C37" s="72"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="72"/>
+      <c r="F37" s="72"/>
+      <c r="G37" s="72"/>
+      <c r="H37" s="72"/>
+      <c r="I37" s="73"/>
     </row>
     <row r="38" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="58" t="s">
+      <c r="B38" s="74" t="s">
         <v>50</v>
       </c>
-      <c r="C38" s="59"/>
-      <c r="D38" s="59"/>
-      <c r="E38" s="59"/>
-      <c r="F38" s="59"/>
-      <c r="G38" s="59"/>
-      <c r="H38" s="59"/>
-      <c r="I38" s="60"/>
+      <c r="C38" s="75"/>
+      <c r="D38" s="75"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="75"/>
+      <c r="G38" s="75"/>
+      <c r="H38" s="75"/>
+      <c r="I38" s="76"/>
     </row>
     <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="64" t="s">
+      <c r="B39" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="C39" s="65"/>
-      <c r="D39" s="65"/>
-      <c r="E39" s="65"/>
-      <c r="F39" s="65"/>
-      <c r="G39" s="65"/>
-      <c r="H39" s="65"/>
-      <c r="I39" s="66"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
+      <c r="G39" s="25"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="26"/>
     </row>
     <row r="40" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="53"/>
-      <c r="C40" s="119"/>
-      <c r="D40" s="119"/>
-      <c r="E40" s="119"/>
-      <c r="F40" s="119"/>
-      <c r="G40" s="119"/>
-      <c r="H40" s="119"/>
-      <c r="I40" s="54"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="22"/>
+      <c r="I40" s="23"/>
     </row>
     <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="53" t="s">
+      <c r="B41" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="C41" s="119"/>
-      <c r="D41" s="119"/>
-      <c r="E41" s="119"/>
-      <c r="F41" s="119"/>
-      <c r="G41" s="119"/>
-      <c r="H41" s="119"/>
-      <c r="I41" s="54"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="23"/>
     </row>
     <row r="42" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="53"/>
-      <c r="C42" s="119"/>
-      <c r="D42" s="119"/>
-      <c r="E42" s="119"/>
-      <c r="F42" s="119"/>
-      <c r="G42" s="119"/>
-      <c r="H42" s="119"/>
-      <c r="I42" s="54"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="23"/>
     </row>
     <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="53" t="s">
+      <c r="B43" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C43" s="119"/>
-      <c r="D43" s="119"/>
-      <c r="E43" s="119"/>
-      <c r="F43" s="119"/>
-      <c r="G43" s="119"/>
-      <c r="H43" s="119"/>
-      <c r="I43" s="54"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="23"/>
     </row>
     <row r="44" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="53"/>
-      <c r="C44" s="119"/>
-      <c r="D44" s="119"/>
-      <c r="E44" s="119"/>
-      <c r="F44" s="119"/>
-      <c r="G44" s="119"/>
-      <c r="H44" s="119"/>
-      <c r="I44" s="54"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="22"/>
+      <c r="I44" s="23"/>
     </row>
     <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B45" s="53" t="s">
+      <c r="B45" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="C45" s="119"/>
-      <c r="D45" s="119"/>
-      <c r="E45" s="119"/>
-      <c r="F45" s="119"/>
-      <c r="G45" s="119"/>
-      <c r="H45" s="119"/>
-      <c r="I45" s="54"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="22"/>
+      <c r="I45" s="23"/>
     </row>
     <row r="46" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="53"/>
-      <c r="C46" s="119"/>
-      <c r="D46" s="119"/>
-      <c r="E46" s="119"/>
-      <c r="F46" s="119"/>
-      <c r="G46" s="119"/>
-      <c r="H46" s="119"/>
-      <c r="I46" s="54"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="23"/>
     </row>
     <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="53" t="s">
+      <c r="B47" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="C47" s="119"/>
-      <c r="D47" s="119"/>
-      <c r="E47" s="119"/>
-      <c r="F47" s="119"/>
-      <c r="G47" s="119"/>
-      <c r="H47" s="119"/>
-      <c r="I47" s="54"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="23"/>
     </row>
     <row r="48" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="53"/>
-      <c r="C48" s="119"/>
-      <c r="D48" s="119"/>
-      <c r="E48" s="119"/>
-      <c r="F48" s="119"/>
-      <c r="G48" s="119"/>
-      <c r="H48" s="119"/>
-      <c r="I48" s="54"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="23"/>
     </row>
     <row r="49" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="53" t="s">
+      <c r="B49" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="C49" s="119"/>
-      <c r="D49" s="119"/>
-      <c r="E49" s="119"/>
-      <c r="F49" s="119"/>
-      <c r="G49" s="119"/>
-      <c r="H49" s="119"/>
-      <c r="I49" s="54"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="22"/>
+      <c r="H49" s="22"/>
+      <c r="I49" s="23"/>
     </row>
     <row r="50" spans="2:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="53" t="s">
+      <c r="B50" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="C50" s="119"/>
-      <c r="D50" s="119"/>
-      <c r="E50" s="119"/>
-      <c r="F50" s="119"/>
-      <c r="G50" s="119"/>
-      <c r="H50" s="119"/>
-      <c r="I50" s="54"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="22"/>
+      <c r="H50" s="22"/>
+      <c r="I50" s="23"/>
     </row>
     <row r="51" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="86" t="s">
+      <c r="B51" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="C51" s="120"/>
-      <c r="D51" s="120"/>
-      <c r="E51" s="120"/>
-      <c r="F51" s="120"/>
-      <c r="G51" s="120"/>
-      <c r="H51" s="120"/>
-      <c r="I51" s="87"/>
+      <c r="C51" s="66"/>
+      <c r="D51" s="66"/>
+      <c r="E51" s="66"/>
+      <c r="F51" s="66"/>
+      <c r="G51" s="66"/>
+      <c r="H51" s="66"/>
+      <c r="I51" s="67"/>
     </row>
     <row r="52" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="115"/>
-      <c r="C52" s="116"/>
-      <c r="D52" s="116"/>
-      <c r="E52" s="116"/>
-      <c r="F52" s="116"/>
-      <c r="G52" s="116"/>
-      <c r="H52" s="116"/>
-      <c r="I52" s="117"/>
+      <c r="B52" s="27"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="28"/>
+      <c r="F52" s="28"/>
+      <c r="G52" s="28"/>
+      <c r="H52" s="28"/>
+      <c r="I52" s="29"/>
     </row>
     <row r="53" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="83" t="s">
+      <c r="B53" s="30" t="s">
         <v>18</v>
       </c>
-      <c r="C53" s="84"/>
-      <c r="D53" s="84"/>
-      <c r="E53" s="84"/>
-      <c r="F53" s="84"/>
-      <c r="G53" s="84"/>
-      <c r="H53" s="84"/>
-      <c r="I53" s="85"/>
+      <c r="C53" s="31"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="31"/>
+      <c r="F53" s="31"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="31"/>
+      <c r="I53" s="32"/>
     </row>
     <row r="54" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="107"/>
-      <c r="C54" s="108"/>
-      <c r="D54" s="108"/>
-      <c r="E54" s="108"/>
-      <c r="F54" s="108"/>
-      <c r="G54" s="108"/>
-      <c r="H54" s="108"/>
-      <c r="I54" s="109"/>
+      <c r="B54" s="12"/>
+      <c r="C54" s="13"/>
+      <c r="D54" s="13"/>
+      <c r="E54" s="13"/>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="13"/>
+      <c r="I54" s="14"/>
     </row>
     <row r="55" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="110"/>
-      <c r="C55" s="121"/>
-      <c r="D55" s="121"/>
-      <c r="E55" s="121"/>
-      <c r="F55" s="121"/>
-      <c r="G55" s="121"/>
-      <c r="H55" s="121"/>
-      <c r="I55" s="111"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+      <c r="G55" s="16"/>
+      <c r="H55" s="16"/>
+      <c r="I55" s="17"/>
     </row>
     <row r="56" spans="2:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="112"/>
-      <c r="C56" s="113"/>
-      <c r="D56" s="113"/>
-      <c r="E56" s="113"/>
-      <c r="F56" s="113"/>
-      <c r="G56" s="113"/>
-      <c r="H56" s="113"/>
-      <c r="I56" s="114"/>
+      <c r="B56" s="18"/>
+      <c r="C56" s="19"/>
+      <c r="D56" s="19"/>
+      <c r="E56" s="19"/>
+      <c r="F56" s="19"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="19"/>
+      <c r="I56" s="20"/>
     </row>
     <row r="57" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="80" t="s">
+      <c r="B57" s="62" t="s">
         <v>53</v>
       </c>
-      <c r="C57" s="81"/>
-      <c r="D57" s="81"/>
-      <c r="E57" s="81"/>
-      <c r="F57" s="81"/>
-      <c r="G57" s="81"/>
-      <c r="H57" s="81"/>
-      <c r="I57" s="82"/>
+      <c r="C57" s="63"/>
+      <c r="D57" s="63"/>
+      <c r="E57" s="63"/>
+      <c r="F57" s="63"/>
+      <c r="G57" s="63"/>
+      <c r="H57" s="63"/>
+      <c r="I57" s="64"/>
     </row>
     <row r="58" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="88" t="s">
+      <c r="B58" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="C58" s="122"/>
-      <c r="D58" s="123" t="s">
+      <c r="C58" s="51"/>
+      <c r="D58" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="E58" s="123"/>
-      <c r="F58" s="123"/>
-      <c r="G58" s="124" t="s">
+      <c r="E58" s="52"/>
+      <c r="F58" s="52"/>
+      <c r="G58" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="H58" s="125"/>
-      <c r="I58" s="28"/>
+      <c r="H58" s="55"/>
+      <c r="I58" s="56"/>
     </row>
     <row r="59" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B59" s="88" t="s">
+      <c r="B59" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="C59" s="122"/>
-      <c r="D59" s="123" t="s">
+      <c r="C59" s="51"/>
+      <c r="D59" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="E59" s="123"/>
-      <c r="F59" s="123"/>
-      <c r="G59" s="124"/>
-      <c r="H59" s="125"/>
-      <c r="I59" s="28"/>
+      <c r="E59" s="52"/>
+      <c r="F59" s="52"/>
+      <c r="G59" s="53"/>
+      <c r="H59" s="55"/>
+      <c r="I59" s="56"/>
     </row>
     <row r="60" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="88"/>
-      <c r="C60" s="122"/>
-      <c r="D60" s="123"/>
-      <c r="E60" s="123"/>
-      <c r="F60" s="123"/>
-      <c r="G60" s="124"/>
-      <c r="H60" s="125"/>
-      <c r="I60" s="28"/>
+      <c r="B60" s="50"/>
+      <c r="C60" s="51"/>
+      <c r="D60" s="52"/>
+      <c r="E60" s="52"/>
+      <c r="F60" s="52"/>
+      <c r="G60" s="53"/>
+      <c r="H60" s="55"/>
+      <c r="I60" s="56"/>
     </row>
     <row r="61" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="89" t="s">
+      <c r="B61" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="C61" s="90"/>
-      <c r="D61" s="90"/>
-      <c r="E61" s="90"/>
-      <c r="F61" s="90"/>
-      <c r="G61" s="90"/>
-      <c r="H61" s="90"/>
-      <c r="I61" s="91"/>
+      <c r="C61" s="48"/>
+      <c r="D61" s="48"/>
+      <c r="E61" s="48"/>
+      <c r="F61" s="48"/>
+      <c r="G61" s="48"/>
+      <c r="H61" s="48"/>
+      <c r="I61" s="49"/>
     </row>
     <row r="62" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="88" t="s">
+      <c r="B62" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="C62" s="122"/>
-      <c r="D62" s="123"/>
-      <c r="E62" s="123"/>
-      <c r="F62" s="123"/>
-      <c r="G62" s="124" t="s">
+      <c r="C62" s="51"/>
+      <c r="D62" s="52"/>
+      <c r="E62" s="52"/>
+      <c r="F62" s="52"/>
+      <c r="G62" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="H62" s="125"/>
-      <c r="I62" s="28"/>
+      <c r="H62" s="55"/>
+      <c r="I62" s="56"/>
     </row>
     <row r="63" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B63" s="88" t="s">
+      <c r="B63" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="C63" s="122"/>
-      <c r="D63" s="123"/>
-      <c r="E63" s="123"/>
-      <c r="F63" s="123"/>
-      <c r="G63" s="124"/>
-      <c r="H63" s="125"/>
-      <c r="I63" s="28"/>
+      <c r="C63" s="51"/>
+      <c r="D63" s="52"/>
+      <c r="E63" s="52"/>
+      <c r="F63" s="52"/>
+      <c r="G63" s="53"/>
+      <c r="H63" s="55"/>
+      <c r="I63" s="56"/>
     </row>
     <row r="64" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="94"/>
-      <c r="C64" s="95"/>
-      <c r="D64" s="96"/>
-      <c r="E64" s="96"/>
-      <c r="F64" s="96"/>
-      <c r="G64" s="92"/>
-      <c r="H64" s="93"/>
-      <c r="I64" s="30"/>
+      <c r="B64" s="59"/>
+      <c r="C64" s="60"/>
+      <c r="D64" s="61"/>
+      <c r="E64" s="61"/>
+      <c r="F64" s="61"/>
+      <c r="G64" s="54"/>
+      <c r="H64" s="57"/>
+      <c r="I64" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="76">
-    <mergeCell ref="B54:I56"/>
-    <mergeCell ref="B49:I49"/>
-    <mergeCell ref="B50:I50"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B39:I40"/>
-    <mergeCell ref="B41:I42"/>
-    <mergeCell ref="B43:I44"/>
-    <mergeCell ref="B45:I46"/>
-    <mergeCell ref="B47:I48"/>
-    <mergeCell ref="B52:I52"/>
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="H20:I22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B61:I61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="D62:F62"/>
-    <mergeCell ref="G62:G64"/>
-    <mergeCell ref="H62:I64"/>
-    <mergeCell ref="B63:C64"/>
-    <mergeCell ref="D63:F64"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="B1:C5"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="D2:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B36:I37"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B7:I9"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B26:I26"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B11:D11"/>
     <mergeCell ref="H58:I60"/>
     <mergeCell ref="B57:I57"/>
     <mergeCell ref="B53:I53"/>
@@ -2595,41 +2597,39 @@
     <mergeCell ref="B29:I29"/>
     <mergeCell ref="B30:I30"/>
     <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B36:I37"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B7:I9"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B26:I26"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B1:C5"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="D2:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="B61:I61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="D62:F62"/>
+    <mergeCell ref="G62:G64"/>
+    <mergeCell ref="H62:I64"/>
+    <mergeCell ref="B63:C64"/>
+    <mergeCell ref="D63:F64"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="H20:I22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B54:I56"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B39:I40"/>
+    <mergeCell ref="B41:I42"/>
+    <mergeCell ref="B43:I44"/>
+    <mergeCell ref="B45:I46"/>
+    <mergeCell ref="B47:I48"/>
+    <mergeCell ref="B52:I52"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.62992125984251968" right="0.23622047244094491" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" scale="58" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.62992125984251968" right="0.62992125984251968" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="55" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="52" min="1" max="8" man="1"/>
   </rowBreaks>
@@ -2640,12 +2640,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="30ba6132-0b50-445c-b091-6b36769966f5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="98b65742-7606-4aba-8ffb-70ac9bc50cd0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2898,20 +2900,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="30ba6132-0b50-445c-b091-6b36769966f5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="98b65742-7606-4aba-8ffb-70ac9bc50cd0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{343F90F2-9DD9-41F8-A266-0D3FA1D7C8B8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="30ba6132-0b50-445c-b091-6b36769966f5"/>
+    <ds:schemaRef ds:uri="98b65742-7606-4aba-8ffb-70ac9bc50cd0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2936,12 +2939,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{343F90F2-9DD9-41F8-A266-0D3FA1D7C8B8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="30ba6132-0b50-445c-b091-6b36769966f5"/>
-    <ds:schemaRef ds:uri="98b65742-7606-4aba-8ffb-70ac9bc50cd0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Modificado filtros y diseño UI
</commit_message>
<xml_diff>
--- a/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
+++ b/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyecto\ControlActivosTI\ControlActivosTI\templates\actas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B121A06-7E1F-4726-BE66-68D2EE067B6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1654EFD5-A8AB-4339-9226-A37017CAD534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13740" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$B$1:$I$64</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$B$1:$I$67</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -114,9 +114,6 @@
     <t>Juan Villacrés</t>
   </si>
   <si>
-    <t>Asistente de TIC'S</t>
-  </si>
-  <si>
     <t>FOTOGRAFÍAS DE LOS EQUIPOS ENTREGADOS</t>
   </si>
   <si>
@@ -463,6 +460,9 @@
   </si>
   <si>
     <t>RECIBE CONFORME (He leído y acepto el contenido del presente documento)</t>
+  </si>
+  <si>
+    <t>ESPECIALISTA DE TIC'S</t>
   </si>
 </sst>
 </file>
@@ -1029,32 +1029,131 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1065,6 +1164,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1074,23 +1200,110 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1099,12 +1312,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1125,250 +1332,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1772,7 +1772,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I64"/>
+  <dimension ref="B1:I67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" style="1" customWidth="1"/>
@@ -1787,166 +1787,166 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="89" t="e" vm="1">
+      <c r="B1" s="25" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="93" t="s">
+      <c r="C1" s="26"/>
+      <c r="D1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="94"/>
-      <c r="F1" s="94"/>
-      <c r="G1" s="95"/>
-      <c r="H1" s="96" t="s">
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="98" t="s">
+      <c r="I1" s="36" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="91"/>
-      <c r="C2" s="56"/>
-      <c r="D2" s="100" t="s">
-        <v>32</v>
-      </c>
-      <c r="E2" s="101"/>
-      <c r="F2" s="101"/>
-      <c r="G2" s="102"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="99"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="38" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="37"/>
     </row>
     <row r="3" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="91"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="104"/>
-      <c r="F3" s="104"/>
-      <c r="G3" s="105"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="28"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="42"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="43"/>
       <c r="H3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="I3" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="27"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
+      <c r="F4" s="42"/>
+      <c r="G4" s="43"/>
+      <c r="H4" s="47" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="49">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="29"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="44"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="48"/>
+      <c r="I5" s="50"/>
+    </row>
+    <row r="6" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="52"/>
+      <c r="D6" s="53"/>
+      <c r="E6" s="75"/>
+      <c r="F6" s="76"/>
+      <c r="G6" s="76"/>
+      <c r="H6" s="76"/>
+      <c r="I6" s="77"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="66" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="91"/>
-      <c r="C4" s="56"/>
-      <c r="D4" s="103"/>
-      <c r="E4" s="104"/>
-      <c r="F4" s="104"/>
-      <c r="G4" s="105"/>
-      <c r="H4" s="109" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="111">
-        <v>46097</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="92"/>
-      <c r="C5" s="58"/>
-      <c r="D5" s="106"/>
-      <c r="E5" s="107"/>
-      <c r="F5" s="107"/>
-      <c r="G5" s="108"/>
-      <c r="H5" s="110"/>
-      <c r="I5" s="112"/>
-    </row>
-    <row r="6" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="68" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="69"/>
-      <c r="D6" s="70"/>
-      <c r="E6" s="84"/>
-      <c r="F6" s="85"/>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="86"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="26"/>
+      <c r="C7" s="67"/>
+      <c r="D7" s="67"/>
+      <c r="E7" s="67"/>
+      <c r="F7" s="67"/>
+      <c r="G7" s="67"/>
+      <c r="H7" s="67"/>
+      <c r="I7" s="68"/>
     </row>
     <row r="8" spans="2:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="21"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="23"/>
+      <c r="B8" s="54"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="56"/>
     </row>
     <row r="9" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="21"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="22"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="23"/>
+      <c r="B9" s="54"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="56"/>
     </row>
     <row r="10" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="124" t="s">
+      <c r="B10" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="19"/>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="80" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="119"/>
-      <c r="D10" s="119"/>
-      <c r="E10" s="125"/>
-      <c r="F10" s="125"/>
-      <c r="G10" s="125"/>
-      <c r="H10" s="119" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="120"/>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="87" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="88"/>
-      <c r="D11" s="88"/>
-      <c r="E11" s="116"/>
-      <c r="F11" s="117"/>
-      <c r="G11" s="118"/>
-      <c r="H11" s="119"/>
-      <c r="I11" s="120"/>
+      <c r="C11" s="81"/>
+      <c r="D11" s="81"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="19"/>
     </row>
     <row r="12" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="121" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" s="122"/>
-      <c r="D12" s="122"/>
-      <c r="E12" s="122"/>
-      <c r="F12" s="122"/>
-      <c r="G12" s="122"/>
-      <c r="H12" s="122"/>
-      <c r="I12" s="123"/>
+      <c r="B12" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="22"/>
     </row>
     <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="78" t="s">
+      <c r="B13" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="79"/>
-      <c r="D13" s="79" t="s">
+      <c r="C13" s="70"/>
+      <c r="D13" s="70" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="79"/>
+      <c r="E13" s="70"/>
       <c r="F13" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>6</v>
@@ -1955,616 +1955,681 @@
         <v>7</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="80"/>
-      <c r="C14" s="77"/>
-      <c r="D14" s="77"/>
-      <c r="E14" s="77"/>
+      <c r="B14" s="71"/>
+      <c r="C14" s="63"/>
+      <c r="D14" s="63"/>
+      <c r="E14" s="63"/>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="9"/>
     </row>
     <row r="15" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="113"/>
-      <c r="C15" s="114"/>
-      <c r="D15" s="115"/>
-      <c r="E15" s="114"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="13"/>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
     </row>
     <row r="16" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="44"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="45"/>
+      <c r="B16" s="78"/>
+      <c r="C16" s="79"/>
+      <c r="D16" s="79"/>
+      <c r="E16" s="79"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="2:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="36"/>
-      <c r="C17" s="37"/>
-      <c r="D17" s="37"/>
-      <c r="E17" s="37"/>
+      <c r="B17" s="64"/>
+      <c r="C17" s="65"/>
+      <c r="D17" s="65"/>
+      <c r="E17" s="65"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="7"/>
     </row>
     <row r="18" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="30" t="s">
+      <c r="B18" s="86" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="87"/>
+      <c r="D18" s="87"/>
+      <c r="E18" s="87"/>
+      <c r="F18" s="87"/>
+      <c r="G18" s="87"/>
+      <c r="H18" s="87"/>
+      <c r="I18" s="88"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="104" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="105"/>
+      <c r="D19" s="105"/>
+      <c r="E19" s="105"/>
+      <c r="F19" s="105" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="105"/>
+      <c r="H19" s="105" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" s="106"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="78" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="79"/>
+      <c r="D20" s="79"/>
+      <c r="E20" s="79"/>
+      <c r="F20" s="113"/>
+      <c r="G20" s="113"/>
+      <c r="H20" s="107" t="s">
+        <v>40</v>
+      </c>
+      <c r="I20" s="108"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="78" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="79"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
+      <c r="F21" s="113"/>
+      <c r="G21" s="113"/>
+      <c r="H21" s="109"/>
+      <c r="I21" s="108"/>
+    </row>
+    <row r="22" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="64" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" s="65"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="112"/>
+      <c r="G22" s="112"/>
+      <c r="H22" s="110"/>
+      <c r="I22" s="111"/>
+    </row>
+    <row r="23" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="72" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="73"/>
+      <c r="D23" s="73"/>
+      <c r="E23" s="73"/>
+      <c r="F23" s="73"/>
+      <c r="G23" s="73"/>
+      <c r="H23" s="73"/>
+      <c r="I23" s="74"/>
+    </row>
+    <row r="24" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="54" t="s">
         <v>45</v>
       </c>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-      <c r="H18" s="31"/>
-      <c r="I18" s="32"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="C19" s="34"/>
-      <c r="D19" s="34"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="34" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="34"/>
-      <c r="H19" s="34" t="s">
-        <v>21</v>
-      </c>
-      <c r="I19" s="35"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="44" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="46"/>
-      <c r="G20" s="46"/>
-      <c r="H20" s="38" t="s">
-        <v>41</v>
-      </c>
-      <c r="I20" s="39"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="44" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21" s="45"/>
-      <c r="D21" s="45"/>
-      <c r="E21" s="45"/>
-      <c r="F21" s="46"/>
-      <c r="G21" s="46"/>
-      <c r="H21" s="40"/>
-      <c r="I21" s="39"/>
-    </row>
-    <row r="22" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="36" t="s">
-        <v>24</v>
-      </c>
-      <c r="C22" s="37"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="37"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="43"/>
-      <c r="H22" s="41"/>
-      <c r="I22" s="42"/>
-    </row>
-    <row r="23" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="81" t="s">
+      <c r="C24" s="55"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="55"/>
+      <c r="F24" s="55"/>
+      <c r="G24" s="55"/>
+      <c r="H24" s="55"/>
+      <c r="I24" s="56"/>
+    </row>
+    <row r="25" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="54"/>
+      <c r="C25" s="55"/>
+      <c r="D25" s="55"/>
+      <c r="E25" s="55"/>
+      <c r="F25" s="55"/>
+      <c r="G25" s="55"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="56"/>
+    </row>
+    <row r="26" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="82"/>
-      <c r="D23" s="82"/>
-      <c r="E23" s="82"/>
-      <c r="F23" s="82"/>
-      <c r="G23" s="82"/>
-      <c r="H23" s="82"/>
-      <c r="I23" s="83"/>
-    </row>
-    <row r="24" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="21" t="s">
+      <c r="C26" s="55"/>
+      <c r="D26" s="55"/>
+      <c r="E26" s="55"/>
+      <c r="F26" s="55"/>
+      <c r="G26" s="55"/>
+      <c r="H26" s="55"/>
+      <c r="I26" s="56"/>
+    </row>
+    <row r="27" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="55"/>
+      <c r="D27" s="55"/>
+      <c r="E27" s="55"/>
+      <c r="F27" s="55"/>
+      <c r="G27" s="55"/>
+      <c r="H27" s="55"/>
+      <c r="I27" s="56"/>
+    </row>
+    <row r="28" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="54" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="55"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="55"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="56"/>
+    </row>
+    <row r="29" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="54" t="s">
+        <v>28</v>
+      </c>
+      <c r="C29" s="55"/>
+      <c r="D29" s="55"/>
+      <c r="E29" s="55"/>
+      <c r="F29" s="55"/>
+      <c r="G29" s="55"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="56"/>
+    </row>
+    <row r="30" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="23"/>
-    </row>
-    <row r="25" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="21"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="23"/>
-    </row>
-    <row r="26" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
-      <c r="I26" s="23"/>
-    </row>
-    <row r="27" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="23"/>
-    </row>
-    <row r="28" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="23"/>
-    </row>
-    <row r="29" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="21" t="s">
+      <c r="C30" s="55"/>
+      <c r="D30" s="55"/>
+      <c r="E30" s="55"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="55"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="56"/>
+    </row>
+    <row r="31" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="54" t="s">
+        <v>47</v>
+      </c>
+      <c r="C31" s="55"/>
+      <c r="D31" s="55"/>
+      <c r="E31" s="55"/>
+      <c r="F31" s="55"/>
+      <c r="G31" s="55"/>
+      <c r="H31" s="55"/>
+      <c r="I31" s="56"/>
+    </row>
+    <row r="32" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="54" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="55"/>
+      <c r="D32" s="55"/>
+      <c r="E32" s="55"/>
+      <c r="F32" s="55"/>
+      <c r="G32" s="55"/>
+      <c r="H32" s="55"/>
+      <c r="I32" s="56"/>
+    </row>
+    <row r="33" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="23"/>
-    </row>
-    <row r="30" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="23"/>
-    </row>
-    <row r="31" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="21" t="s">
+      <c r="C33" s="55"/>
+      <c r="D33" s="55"/>
+      <c r="E33" s="55"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="55"/>
+      <c r="H33" s="55"/>
+      <c r="I33" s="56"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B34" s="54" t="s">
         <v>48</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="22"/>
-      <c r="E31" s="22"/>
-      <c r="F31" s="22"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="22"/>
-      <c r="I31" s="23"/>
-    </row>
-    <row r="32" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="22"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="23"/>
-    </row>
-    <row r="33" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="21" t="s">
+      <c r="C34" s="55"/>
+      <c r="D34" s="55"/>
+      <c r="E34" s="55"/>
+      <c r="F34" s="55"/>
+      <c r="G34" s="55"/>
+      <c r="H34" s="55"/>
+      <c r="I34" s="56"/>
+    </row>
+    <row r="35" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="54"/>
+      <c r="C35" s="55"/>
+      <c r="D35" s="55"/>
+      <c r="E35" s="55"/>
+      <c r="F35" s="55"/>
+      <c r="G35" s="55"/>
+      <c r="H35" s="55"/>
+      <c r="I35" s="56"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B36" s="54" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="55"/>
+      <c r="D36" s="55"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="55"/>
+      <c r="H36" s="55"/>
+      <c r="I36" s="56"/>
+    </row>
+    <row r="37" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="57"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="58"/>
+      <c r="E37" s="58"/>
+      <c r="F37" s="58"/>
+      <c r="G37" s="58"/>
+      <c r="H37" s="58"/>
+      <c r="I37" s="59"/>
+    </row>
+    <row r="38" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="60" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
+      <c r="G38" s="61"/>
+      <c r="H38" s="61"/>
+      <c r="I38" s="62"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B39" s="66" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="67"/>
+      <c r="D39" s="67"/>
+      <c r="E39" s="67"/>
+      <c r="F39" s="67"/>
+      <c r="G39" s="67"/>
+      <c r="H39" s="67"/>
+      <c r="I39" s="68"/>
+    </row>
+    <row r="40" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="54"/>
+      <c r="C40" s="55"/>
+      <c r="D40" s="55"/>
+      <c r="E40" s="55"/>
+      <c r="F40" s="55"/>
+      <c r="G40" s="55"/>
+      <c r="H40" s="55"/>
+      <c r="I40" s="56"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="55"/>
+      <c r="D41" s="55"/>
+      <c r="E41" s="55"/>
+      <c r="F41" s="55"/>
+      <c r="G41" s="55"/>
+      <c r="H41" s="55"/>
+      <c r="I41" s="56"/>
+    </row>
+    <row r="42" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="54"/>
+      <c r="C42" s="55"/>
+      <c r="D42" s="55"/>
+      <c r="E42" s="55"/>
+      <c r="F42" s="55"/>
+      <c r="G42" s="55"/>
+      <c r="H42" s="55"/>
+      <c r="I42" s="56"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="54" t="s">
+        <v>50</v>
+      </c>
+      <c r="C43" s="55"/>
+      <c r="D43" s="55"/>
+      <c r="E43" s="55"/>
+      <c r="F43" s="55"/>
+      <c r="G43" s="55"/>
+      <c r="H43" s="55"/>
+      <c r="I43" s="56"/>
+    </row>
+    <row r="44" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="54"/>
+      <c r="C44" s="55"/>
+      <c r="D44" s="55"/>
+      <c r="E44" s="55"/>
+      <c r="F44" s="55"/>
+      <c r="G44" s="55"/>
+      <c r="H44" s="55"/>
+      <c r="I44" s="56"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45" s="54" t="s">
+        <v>51</v>
+      </c>
+      <c r="C45" s="55"/>
+      <c r="D45" s="55"/>
+      <c r="E45" s="55"/>
+      <c r="F45" s="55"/>
+      <c r="G45" s="55"/>
+      <c r="H45" s="55"/>
+      <c r="I45" s="56"/>
+    </row>
+    <row r="46" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="54"/>
+      <c r="C46" s="55"/>
+      <c r="D46" s="55"/>
+      <c r="E46" s="55"/>
+      <c r="F46" s="55"/>
+      <c r="G46" s="55"/>
+      <c r="H46" s="55"/>
+      <c r="I46" s="56"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="54" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="55"/>
+      <c r="D47" s="55"/>
+      <c r="E47" s="55"/>
+      <c r="F47" s="55"/>
+      <c r="G47" s="55"/>
+      <c r="H47" s="55"/>
+      <c r="I47" s="56"/>
+    </row>
+    <row r="48" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="54"/>
+      <c r="C48" s="55"/>
+      <c r="D48" s="55"/>
+      <c r="E48" s="55"/>
+      <c r="F48" s="55"/>
+      <c r="G48" s="55"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="56"/>
+    </row>
+    <row r="49" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="54" t="s">
+        <v>34</v>
+      </c>
+      <c r="C49" s="55"/>
+      <c r="D49" s="55"/>
+      <c r="E49" s="55"/>
+      <c r="F49" s="55"/>
+      <c r="G49" s="55"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="56"/>
+    </row>
+    <row r="50" spans="2:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="54" t="s">
+        <v>35</v>
+      </c>
+      <c r="C50" s="55"/>
+      <c r="D50" s="55"/>
+      <c r="E50" s="55"/>
+      <c r="F50" s="55"/>
+      <c r="G50" s="55"/>
+      <c r="H50" s="55"/>
+      <c r="I50" s="56"/>
+    </row>
+    <row r="51" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="22"/>
-      <c r="D33" s="22"/>
-      <c r="E33" s="22"/>
-      <c r="F33" s="22"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="22"/>
-      <c r="I33" s="23"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C34" s="22"/>
-      <c r="D34" s="22"/>
-      <c r="E34" s="22"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="23"/>
-    </row>
-    <row r="35" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="21"/>
-      <c r="C35" s="22"/>
-      <c r="D35" s="22"/>
-      <c r="E35" s="22"/>
-      <c r="F35" s="22"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22"/>
-      <c r="I35" s="23"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="22"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="23"/>
-    </row>
-    <row r="37" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="71"/>
-      <c r="C37" s="72"/>
-      <c r="D37" s="72"/>
-      <c r="E37" s="72"/>
-      <c r="F37" s="72"/>
-      <c r="G37" s="72"/>
-      <c r="H37" s="72"/>
-      <c r="I37" s="73"/>
-    </row>
-    <row r="38" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="74" t="s">
-        <v>50</v>
-      </c>
-      <c r="C38" s="75"/>
-      <c r="D38" s="75"/>
-      <c r="E38" s="75"/>
-      <c r="F38" s="75"/>
-      <c r="G38" s="75"/>
-      <c r="H38" s="75"/>
-      <c r="I38" s="76"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="C39" s="25"/>
-      <c r="D39" s="25"/>
-      <c r="E39" s="25"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="26"/>
-    </row>
-    <row r="40" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="21"/>
-      <c r="C40" s="22"/>
-      <c r="D40" s="22"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="22"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="23"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="21" t="s">
-        <v>11</v>
-      </c>
-      <c r="C41" s="22"/>
-      <c r="D41" s="22"/>
-      <c r="E41" s="22"/>
-      <c r="F41" s="22"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="23"/>
-    </row>
-    <row r="42" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="21"/>
-      <c r="C42" s="22"/>
-      <c r="D42" s="22"/>
-      <c r="E42" s="22"/>
-      <c r="F42" s="22"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="23"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="C43" s="22"/>
-      <c r="D43" s="22"/>
-      <c r="E43" s="22"/>
-      <c r="F43" s="22"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="22"/>
-      <c r="I43" s="23"/>
-    </row>
-    <row r="44" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="21"/>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="22"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="22"/>
-      <c r="I44" s="23"/>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B45" s="21" t="s">
+      <c r="C51" s="90"/>
+      <c r="D51" s="90"/>
+      <c r="E51" s="90"/>
+      <c r="F51" s="90"/>
+      <c r="G51" s="90"/>
+      <c r="H51" s="90"/>
+      <c r="I51" s="91"/>
+    </row>
+    <row r="52" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="122"/>
+      <c r="C52" s="123"/>
+      <c r="D52" s="123"/>
+      <c r="E52" s="123"/>
+      <c r="F52" s="123"/>
+      <c r="G52" s="123"/>
+      <c r="H52" s="123"/>
+      <c r="I52" s="124"/>
+    </row>
+    <row r="53" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="86" t="s">
+        <v>17</v>
+      </c>
+      <c r="C53" s="87"/>
+      <c r="D53" s="87"/>
+      <c r="E53" s="87"/>
+      <c r="F53" s="87"/>
+      <c r="G53" s="87"/>
+      <c r="H53" s="87"/>
+      <c r="I53" s="88"/>
+    </row>
+    <row r="54" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="114"/>
+      <c r="C54" s="115"/>
+      <c r="D54" s="115"/>
+      <c r="E54" s="115"/>
+      <c r="F54" s="115"/>
+      <c r="G54" s="115"/>
+      <c r="H54" s="115"/>
+      <c r="I54" s="116"/>
+    </row>
+    <row r="55" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="117"/>
+      <c r="C55" s="125"/>
+      <c r="D55" s="125"/>
+      <c r="E55" s="125"/>
+      <c r="F55" s="125"/>
+      <c r="G55" s="125"/>
+      <c r="H55" s="125"/>
+      <c r="I55" s="118"/>
+    </row>
+    <row r="56" spans="2:9" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="117"/>
+      <c r="C56" s="125"/>
+      <c r="D56" s="125"/>
+      <c r="E56" s="125"/>
+      <c r="F56" s="125"/>
+      <c r="G56" s="125"/>
+      <c r="H56" s="125"/>
+      <c r="I56" s="118"/>
+    </row>
+    <row r="57" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="117"/>
+      <c r="C57" s="125"/>
+      <c r="D57" s="125"/>
+      <c r="E57" s="125"/>
+      <c r="F57" s="125"/>
+      <c r="G57" s="125"/>
+      <c r="H57" s="125"/>
+      <c r="I57" s="118"/>
+    </row>
+    <row r="58" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="117"/>
+      <c r="C58" s="125"/>
+      <c r="D58" s="125"/>
+      <c r="E58" s="125"/>
+      <c r="F58" s="125"/>
+      <c r="G58" s="125"/>
+      <c r="H58" s="125"/>
+      <c r="I58" s="118"/>
+    </row>
+    <row r="59" spans="2:9" ht="89.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="119"/>
+      <c r="C59" s="120"/>
+      <c r="D59" s="120"/>
+      <c r="E59" s="120"/>
+      <c r="F59" s="120"/>
+      <c r="G59" s="120"/>
+      <c r="H59" s="120"/>
+      <c r="I59" s="121"/>
+    </row>
+    <row r="60" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="83" t="s">
         <v>52</v>
       </c>
-      <c r="C45" s="22"/>
-      <c r="D45" s="22"/>
-      <c r="E45" s="22"/>
-      <c r="F45" s="22"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="22"/>
-      <c r="I45" s="23"/>
-    </row>
-    <row r="46" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="21"/>
-      <c r="C46" s="22"/>
-      <c r="D46" s="22"/>
-      <c r="E46" s="22"/>
-      <c r="F46" s="22"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="23"/>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="C47" s="22"/>
-      <c r="D47" s="22"/>
-      <c r="E47" s="22"/>
-      <c r="F47" s="22"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="22"/>
-      <c r="I47" s="23"/>
-    </row>
-    <row r="48" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="21"/>
-      <c r="C48" s="22"/>
-      <c r="D48" s="22"/>
-      <c r="E48" s="22"/>
-      <c r="F48" s="22"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="23"/>
-    </row>
-    <row r="49" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="C49" s="22"/>
-      <c r="D49" s="22"/>
-      <c r="E49" s="22"/>
-      <c r="F49" s="22"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="22"/>
-      <c r="I49" s="23"/>
-    </row>
-    <row r="50" spans="2:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C50" s="22"/>
-      <c r="D50" s="22"/>
-      <c r="E50" s="22"/>
-      <c r="F50" s="22"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="22"/>
-      <c r="I50" s="23"/>
-    </row>
-    <row r="51" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="65" t="s">
-        <v>31</v>
-      </c>
-      <c r="C51" s="66"/>
-      <c r="D51" s="66"/>
-      <c r="E51" s="66"/>
-      <c r="F51" s="66"/>
-      <c r="G51" s="66"/>
-      <c r="H51" s="66"/>
-      <c r="I51" s="67"/>
-    </row>
-    <row r="52" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="27"/>
-      <c r="C52" s="28"/>
-      <c r="D52" s="28"/>
-      <c r="E52" s="28"/>
-      <c r="F52" s="28"/>
-      <c r="G52" s="28"/>
-      <c r="H52" s="28"/>
-      <c r="I52" s="29"/>
-    </row>
-    <row r="53" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="30" t="s">
-        <v>18</v>
-      </c>
-      <c r="C53" s="31"/>
-      <c r="D53" s="31"/>
-      <c r="E53" s="31"/>
-      <c r="F53" s="31"/>
-      <c r="G53" s="31"/>
-      <c r="H53" s="31"/>
-      <c r="I53" s="32"/>
-    </row>
-    <row r="54" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="12"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="13"/>
-      <c r="H54" s="13"/>
-      <c r="I54" s="14"/>
-    </row>
-    <row r="55" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="15"/>
-      <c r="C55" s="16"/>
-      <c r="D55" s="16"/>
-      <c r="E55" s="16"/>
-      <c r="F55" s="16"/>
-      <c r="G55" s="16"/>
-      <c r="H55" s="16"/>
-      <c r="I55" s="17"/>
-    </row>
-    <row r="56" spans="2:9" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="18"/>
-      <c r="C56" s="19"/>
-      <c r="D56" s="19"/>
-      <c r="E56" s="19"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="19"/>
-      <c r="I56" s="20"/>
-    </row>
-    <row r="57" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="62" t="s">
+      <c r="C60" s="84"/>
+      <c r="D60" s="84"/>
+      <c r="E60" s="84"/>
+      <c r="F60" s="84"/>
+      <c r="G60" s="84"/>
+      <c r="H60" s="84"/>
+      <c r="I60" s="85"/>
+    </row>
+    <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="93" t="s">
+        <v>13</v>
+      </c>
+      <c r="C61" s="94"/>
+      <c r="D61" s="92" t="s">
+        <v>16</v>
+      </c>
+      <c r="E61" s="92"/>
+      <c r="F61" s="92"/>
+      <c r="G61" s="95" t="s">
+        <v>15</v>
+      </c>
+      <c r="H61" s="82"/>
+      <c r="I61" s="28"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B62" s="93" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62" s="94"/>
+      <c r="D62" s="92" t="s">
+        <v>54</v>
+      </c>
+      <c r="E62" s="92"/>
+      <c r="F62" s="92"/>
+      <c r="G62" s="95"/>
+      <c r="H62" s="82"/>
+      <c r="I62" s="28"/>
+    </row>
+    <row r="63" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="93"/>
+      <c r="C63" s="94"/>
+      <c r="D63" s="92"/>
+      <c r="E63" s="92"/>
+      <c r="F63" s="92"/>
+      <c r="G63" s="95"/>
+      <c r="H63" s="82"/>
+      <c r="I63" s="28"/>
+    </row>
+    <row r="64" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B64" s="96" t="s">
         <v>53</v>
       </c>
-      <c r="C57" s="63"/>
-      <c r="D57" s="63"/>
-      <c r="E57" s="63"/>
-      <c r="F57" s="63"/>
-      <c r="G57" s="63"/>
-      <c r="H57" s="63"/>
-      <c r="I57" s="64"/>
-    </row>
-    <row r="58" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="50" t="s">
+      <c r="C64" s="97"/>
+      <c r="D64" s="97"/>
+      <c r="E64" s="97"/>
+      <c r="F64" s="97"/>
+      <c r="G64" s="97"/>
+      <c r="H64" s="97"/>
+      <c r="I64" s="98"/>
+    </row>
+    <row r="65" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="93" t="s">
         <v>13</v>
       </c>
-      <c r="C58" s="51"/>
-      <c r="D58" s="52" t="s">
-        <v>16</v>
-      </c>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="53" t="s">
+      <c r="C65" s="94"/>
+      <c r="D65" s="92"/>
+      <c r="E65" s="92"/>
+      <c r="F65" s="92"/>
+      <c r="G65" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="H58" s="55"/>
-      <c r="I58" s="56"/>
-    </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B59" s="50" t="s">
+      <c r="H65" s="82"/>
+      <c r="I65" s="28"/>
+    </row>
+    <row r="66" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B66" s="93" t="s">
         <v>14</v>
       </c>
-      <c r="C59" s="51"/>
-      <c r="D59" s="52" t="s">
-        <v>17</v>
-      </c>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="53"/>
-      <c r="H59" s="55"/>
-      <c r="I59" s="56"/>
-    </row>
-    <row r="60" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="50"/>
-      <c r="C60" s="51"/>
-      <c r="D60" s="52"/>
-      <c r="E60" s="52"/>
-      <c r="F60" s="52"/>
-      <c r="G60" s="53"/>
-      <c r="H60" s="55"/>
-      <c r="I60" s="56"/>
-    </row>
-    <row r="61" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="47" t="s">
-        <v>54</v>
-      </c>
-      <c r="C61" s="48"/>
-      <c r="D61" s="48"/>
-      <c r="E61" s="48"/>
-      <c r="F61" s="48"/>
-      <c r="G61" s="48"/>
-      <c r="H61" s="48"/>
-      <c r="I61" s="49"/>
-    </row>
-    <row r="62" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B62" s="50" t="s">
-        <v>13</v>
-      </c>
-      <c r="C62" s="51"/>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="53" t="s">
-        <v>15</v>
-      </c>
-      <c r="H62" s="55"/>
-      <c r="I62" s="56"/>
-    </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B63" s="50" t="s">
-        <v>14</v>
-      </c>
-      <c r="C63" s="51"/>
-      <c r="D63" s="52"/>
-      <c r="E63" s="52"/>
-      <c r="F63" s="52"/>
-      <c r="G63" s="53"/>
-      <c r="H63" s="55"/>
-      <c r="I63" s="56"/>
-    </row>
-    <row r="64" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="59"/>
-      <c r="C64" s="60"/>
-      <c r="D64" s="61"/>
-      <c r="E64" s="61"/>
-      <c r="F64" s="61"/>
-      <c r="G64" s="54"/>
-      <c r="H64" s="57"/>
-      <c r="I64" s="58"/>
+      <c r="C66" s="94"/>
+      <c r="D66" s="92"/>
+      <c r="E66" s="92"/>
+      <c r="F66" s="92"/>
+      <c r="G66" s="95"/>
+      <c r="H66" s="82"/>
+      <c r="I66" s="28"/>
+    </row>
+    <row r="67" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="101"/>
+      <c r="C67" s="102"/>
+      <c r="D67" s="103"/>
+      <c r="E67" s="103"/>
+      <c r="F67" s="103"/>
+      <c r="G67" s="99"/>
+      <c r="H67" s="100"/>
+      <c r="I67" s="30"/>
     </row>
   </sheetData>
-  <mergeCells count="76">
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="B1:C5"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="D2:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
+  <mergeCells count="81">
+    <mergeCell ref="B57:D59"/>
+    <mergeCell ref="E54:G56"/>
+    <mergeCell ref="E57:G59"/>
+    <mergeCell ref="H54:I56"/>
+    <mergeCell ref="H57:I59"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B39:I40"/>
+    <mergeCell ref="B41:I42"/>
+    <mergeCell ref="B43:I44"/>
+    <mergeCell ref="B45:I46"/>
+    <mergeCell ref="B47:I48"/>
+    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B54:D56"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="H20:I22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="G65:G67"/>
+    <mergeCell ref="H65:I67"/>
+    <mergeCell ref="B66:C67"/>
+    <mergeCell ref="D66:F67"/>
+    <mergeCell ref="H61:I63"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="B24:I25"/>
+    <mergeCell ref="B34:I35"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="D61:F61"/>
+    <mergeCell ref="B62:C63"/>
+    <mergeCell ref="D62:F63"/>
+    <mergeCell ref="G61:G63"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B31:I31"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B36:I37"/>
     <mergeCell ref="B38:I38"/>
@@ -2581,52 +2646,27 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="B11:D11"/>
-    <mergeCell ref="H58:I60"/>
-    <mergeCell ref="B57:I57"/>
-    <mergeCell ref="B53:I53"/>
-    <mergeCell ref="B24:I25"/>
-    <mergeCell ref="B34:I35"/>
-    <mergeCell ref="B51:I51"/>
-    <mergeCell ref="D58:F58"/>
-    <mergeCell ref="B59:C60"/>
-    <mergeCell ref="D59:F60"/>
-    <mergeCell ref="G58:G60"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B27:I27"/>
-    <mergeCell ref="B28:I28"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B61:I61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="D62:F62"/>
-    <mergeCell ref="G62:G64"/>
-    <mergeCell ref="H62:I64"/>
-    <mergeCell ref="B63:C64"/>
-    <mergeCell ref="D63:F64"/>
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="H20:I22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B54:I56"/>
-    <mergeCell ref="B49:I49"/>
-    <mergeCell ref="B50:I50"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B39:I40"/>
-    <mergeCell ref="B41:I42"/>
-    <mergeCell ref="B43:I44"/>
-    <mergeCell ref="B45:I46"/>
-    <mergeCell ref="B47:I48"/>
-    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B1:C5"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="D2:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:G10"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G14:G17" xr:uid="{C164E967-E733-492B-B646-A77CBB30BFA0}">
+      <formula1>"NUEVO,FUNCIONAL"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.62992125984251968" right="0.62992125984251968" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="55" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -2640,14 +2680,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="30ba6132-0b50-445c-b091-6b36769966f5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="98b65742-7606-4aba-8ffb-70ac9bc50cd0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2900,21 +2938,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="30ba6132-0b50-445c-b091-6b36769966f5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="98b65742-7606-4aba-8ffb-70ac9bc50cd0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{343F90F2-9DD9-41F8-A266-0D3FA1D7C8B8}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="30ba6132-0b50-445c-b091-6b36769966f5"/>
-    <ds:schemaRef ds:uri="98b65742-7606-4aba-8ffb-70ac9bc50cd0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2939,9 +2976,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{343F90F2-9DD9-41F8-A266-0D3FA1D7C8B8}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="30ba6132-0b50-445c-b091-6b36769966f5"/>
+    <ds:schemaRef ds:uri="98b65742-7606-4aba-8ffb-70ac9bc50cd0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Corregido formato de actas
</commit_message>
<xml_diff>
--- a/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
+++ b/ControlActivosTI/templates/actas/1. F-TI-01 - Acta de Asignación y Entrega de Equipos y Servicios de Tecnología.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyecto\ControlActivosTI\ControlActivosTI\templates\actas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1654EFD5-A8AB-4339-9226-A37017CAD534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D76FA45-B9AB-4B4B-8C49-5436C87E57F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{109ABBD4-A228-4D84-8C4A-06D4C971BB15}"/>
   </bookViews>
@@ -111,9 +111,6 @@
     <t>Firma</t>
   </si>
   <si>
-    <t>Juan Villacrés</t>
-  </si>
-  <si>
     <t>FOTOGRAFÍAS DE LOS EQUIPOS ENTREGADOS</t>
   </si>
   <si>
@@ -463,6 +460,9 @@
   </si>
   <si>
     <t>ESPECIALISTA DE TIC'S</t>
+  </si>
+  <si>
+    <t>JUAN VILLACRÉS</t>
   </si>
 </sst>
 </file>
@@ -1029,6 +1029,309 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1066,309 +1369,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1787,166 +1787,166 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="25" t="e" vm="1">
+      <c r="B1" s="89" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="31" t="s">
+      <c r="C1" s="90"/>
+      <c r="D1" s="93" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="34" t="s">
+      <c r="E1" s="94"/>
+      <c r="F1" s="94"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="I1" s="36" t="s">
+      <c r="I1" s="98" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="27"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="37"/>
+      <c r="B2" s="91"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="100" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="101"/>
+      <c r="F2" s="101"/>
+      <c r="G2" s="102"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="99"/>
     </row>
     <row r="3" spans="2:9" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="27"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="43"/>
+      <c r="B3" s="91"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="104"/>
+      <c r="F3" s="104"/>
+      <c r="G3" s="105"/>
       <c r="H3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="I3" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="91"/>
+      <c r="C4" s="56"/>
+      <c r="D4" s="103"/>
+      <c r="E4" s="104"/>
+      <c r="F4" s="104"/>
+      <c r="G4" s="105"/>
+      <c r="H4" s="109" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="111">
+        <v>46097</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="92"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="106"/>
+      <c r="E5" s="107"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="108"/>
+      <c r="H5" s="110"/>
+      <c r="I5" s="112"/>
+    </row>
+    <row r="6" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="68" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="69"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="84"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
+      <c r="I6" s="86"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="23" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="4" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="27"/>
-      <c r="C4" s="28"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="47" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="49">
-        <v>46097</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="29"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="44"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46"/>
-      <c r="H5" s="48"/>
-      <c r="I5" s="50"/>
-    </row>
-    <row r="6" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="51" t="s">
-        <v>41</v>
-      </c>
-      <c r="C6" s="52"/>
-      <c r="D6" s="53"/>
-      <c r="E6" s="75"/>
-      <c r="F6" s="76"/>
-      <c r="G6" s="76"/>
-      <c r="H6" s="76"/>
-      <c r="I6" s="77"/>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B7" s="66" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
-      <c r="G7" s="67"/>
-      <c r="H7" s="67"/>
-      <c r="I7" s="68"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="25"/>
     </row>
     <row r="8" spans="2:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="54"/>
-      <c r="C8" s="55"/>
-      <c r="D8" s="55"/>
-      <c r="E8" s="55"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="56"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="22"/>
     </row>
     <row r="9" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="54"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="55"/>
-      <c r="E9" s="55"/>
-      <c r="F9" s="55"/>
-      <c r="G9" s="55"/>
-      <c r="H9" s="55"/>
-      <c r="I9" s="56"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="22"/>
     </row>
     <row r="10" spans="2:9" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="124" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="119"/>
+      <c r="D10" s="119"/>
+      <c r="E10" s="125"/>
+      <c r="F10" s="125"/>
+      <c r="G10" s="125"/>
+      <c r="H10" s="119" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="120"/>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="87" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="19"/>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="80" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="81"/>
-      <c r="D11" s="81"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="19"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="116"/>
+      <c r="F11" s="117"/>
+      <c r="G11" s="118"/>
+      <c r="H11" s="119"/>
+      <c r="I11" s="120"/>
     </row>
     <row r="12" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="22"/>
+      <c r="B12" s="121" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="122"/>
+      <c r="D12" s="122"/>
+      <c r="E12" s="122"/>
+      <c r="F12" s="122"/>
+      <c r="G12" s="122"/>
+      <c r="H12" s="122"/>
+      <c r="I12" s="123"/>
     </row>
     <row r="13" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="69" t="s">
+      <c r="B13" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="70"/>
-      <c r="D13" s="70" t="s">
+      <c r="C13" s="79"/>
+      <c r="D13" s="79" t="s">
         <v>5</v>
       </c>
-      <c r="E13" s="70"/>
+      <c r="E13" s="79"/>
       <c r="F13" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>6</v>
@@ -1955,665 +1955,662 @@
         <v>7</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="71"/>
-      <c r="C14" s="63"/>
-      <c r="D14" s="63"/>
-      <c r="E14" s="63"/>
+      <c r="B14" s="80"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
       <c r="I14" s="9"/>
     </row>
     <row r="15" spans="2:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="13"/>
+      <c r="B15" s="113"/>
+      <c r="C15" s="114"/>
+      <c r="D15" s="115"/>
+      <c r="E15" s="114"/>
       <c r="F15" s="8"/>
       <c r="G15" s="8"/>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
     </row>
     <row r="16" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="78"/>
-      <c r="C16" s="79"/>
-      <c r="D16" s="79"/>
-      <c r="E16" s="79"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
       <c r="H16" s="5"/>
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="2:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="64"/>
-      <c r="C17" s="65"/>
-      <c r="D17" s="65"/>
-      <c r="E17" s="65"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
       <c r="F17" s="6"/>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="I17" s="7"/>
     </row>
     <row r="18" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="86" t="s">
+      <c r="B18" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="31"/>
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+      <c r="I18" s="32"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34" t="s">
+        <v>19</v>
+      </c>
+      <c r="I19" s="35"/>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="44" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="46"/>
+      <c r="G20" s="46"/>
+      <c r="H20" s="38" t="s">
+        <v>39</v>
+      </c>
+      <c r="I20" s="39"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="45"/>
+      <c r="D21" s="45"/>
+      <c r="E21" s="45"/>
+      <c r="F21" s="46"/>
+      <c r="G21" s="46"/>
+      <c r="H21" s="40"/>
+      <c r="I21" s="39"/>
+    </row>
+    <row r="22" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="43"/>
+      <c r="G22" s="43"/>
+      <c r="H22" s="41"/>
+      <c r="I22" s="42"/>
+    </row>
+    <row r="23" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="81" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="82"/>
+      <c r="D23" s="82"/>
+      <c r="E23" s="82"/>
+      <c r="F23" s="82"/>
+      <c r="G23" s="82"/>
+      <c r="H23" s="82"/>
+      <c r="I23" s="83"/>
+    </row>
+    <row r="24" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="87"/>
-      <c r="D18" s="87"/>
-      <c r="E18" s="87"/>
-      <c r="F18" s="87"/>
-      <c r="G18" s="87"/>
-      <c r="H18" s="87"/>
-      <c r="I18" s="88"/>
-    </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B19" s="104" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="105"/>
-      <c r="D19" s="105"/>
-      <c r="E19" s="105"/>
-      <c r="F19" s="105" t="s">
-        <v>19</v>
-      </c>
-      <c r="G19" s="105"/>
-      <c r="H19" s="105" t="s">
-        <v>20</v>
-      </c>
-      <c r="I19" s="106"/>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B20" s="78" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="79"/>
-      <c r="D20" s="79"/>
-      <c r="E20" s="79"/>
-      <c r="F20" s="113"/>
-      <c r="G20" s="113"/>
-      <c r="H20" s="107" t="s">
-        <v>40</v>
-      </c>
-      <c r="I20" s="108"/>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B21" s="78" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="79"/>
-      <c r="D21" s="79"/>
-      <c r="E21" s="79"/>
-      <c r="F21" s="113"/>
-      <c r="G21" s="113"/>
-      <c r="H21" s="109"/>
-      <c r="I21" s="108"/>
-    </row>
-    <row r="22" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="64" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="65"/>
-      <c r="D22" s="65"/>
-      <c r="E22" s="65"/>
-      <c r="F22" s="112"/>
-      <c r="G22" s="112"/>
-      <c r="H22" s="110"/>
-      <c r="I22" s="111"/>
-    </row>
-    <row r="23" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="72" t="s">
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="21"/>
+      <c r="H24" s="21"/>
+      <c r="I24" s="22"/>
+    </row>
+    <row r="25" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="20"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="22"/>
+    </row>
+    <row r="26" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="C23" s="73"/>
-      <c r="D23" s="73"/>
-      <c r="E23" s="73"/>
-      <c r="F23" s="73"/>
-      <c r="G23" s="73"/>
-      <c r="H23" s="73"/>
-      <c r="I23" s="74"/>
-    </row>
-    <row r="24" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="54" t="s">
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="21"/>
+      <c r="H26" s="21"/>
+      <c r="I26" s="22"/>
+    </row>
+    <row r="27" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="21"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="22"/>
+    </row>
+    <row r="28" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="22"/>
+    </row>
+    <row r="29" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="21"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="21"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="22"/>
+    </row>
+    <row r="30" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
-      <c r="E24" s="55"/>
-      <c r="F24" s="55"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="55"/>
-      <c r="I24" s="56"/>
-    </row>
-    <row r="25" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="54"/>
-      <c r="C25" s="55"/>
-      <c r="D25" s="55"/>
-      <c r="E25" s="55"/>
-      <c r="F25" s="55"/>
-      <c r="G25" s="55"/>
-      <c r="H25" s="55"/>
-      <c r="I25" s="56"/>
-    </row>
-    <row r="26" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="54" t="s">
-        <v>25</v>
-      </c>
-      <c r="C26" s="55"/>
-      <c r="D26" s="55"/>
-      <c r="E26" s="55"/>
-      <c r="F26" s="55"/>
-      <c r="G26" s="55"/>
-      <c r="H26" s="55"/>
-      <c r="I26" s="56"/>
-    </row>
-    <row r="27" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="55"/>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="55"/>
-      <c r="G27" s="55"/>
-      <c r="H27" s="55"/>
-      <c r="I27" s="56"/>
-    </row>
-    <row r="28" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="C28" s="55"/>
-      <c r="D28" s="55"/>
-      <c r="E28" s="55"/>
-      <c r="F28" s="55"/>
-      <c r="G28" s="55"/>
-      <c r="H28" s="55"/>
-      <c r="I28" s="56"/>
-    </row>
-    <row r="29" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="54" t="s">
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="21"/>
+      <c r="H30" s="21"/>
+      <c r="I30" s="22"/>
+    </row>
+    <row r="31" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="21"/>
+      <c r="H31" s="21"/>
+      <c r="I31" s="22"/>
+    </row>
+    <row r="32" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="22"/>
+    </row>
+    <row r="33" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="55"/>
-      <c r="I29" s="56"/>
-    </row>
-    <row r="30" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="54" t="s">
-        <v>46</v>
-      </c>
-      <c r="C30" s="55"/>
-      <c r="D30" s="55"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="55"/>
-      <c r="H30" s="55"/>
-      <c r="I30" s="56"/>
-    </row>
-    <row r="31" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="54" t="s">
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="22"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B34" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="C31" s="55"/>
-      <c r="D31" s="55"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="55"/>
-      <c r="G31" s="55"/>
-      <c r="H31" s="55"/>
-      <c r="I31" s="56"/>
-    </row>
-    <row r="32" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="54" t="s">
-        <v>38</v>
-      </c>
-      <c r="C32" s="55"/>
-      <c r="D32" s="55"/>
-      <c r="E32" s="55"/>
-      <c r="F32" s="55"/>
-      <c r="G32" s="55"/>
-      <c r="H32" s="55"/>
-      <c r="I32" s="56"/>
-    </row>
-    <row r="33" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="54" t="s">
+      <c r="C34" s="21"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="21"/>
+      <c r="H34" s="21"/>
+      <c r="I34" s="22"/>
+    </row>
+    <row r="35" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="20"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="21"/>
+      <c r="H35" s="21"/>
+      <c r="I35" s="22"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B36" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="22"/>
+    </row>
+    <row r="37" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="71"/>
+      <c r="C37" s="72"/>
+      <c r="D37" s="72"/>
+      <c r="E37" s="72"/>
+      <c r="F37" s="72"/>
+      <c r="G37" s="72"/>
+      <c r="H37" s="72"/>
+      <c r="I37" s="73"/>
+    </row>
+    <row r="38" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="74" t="s">
+        <v>48</v>
+      </c>
+      <c r="C38" s="75"/>
+      <c r="D38" s="75"/>
+      <c r="E38" s="75"/>
+      <c r="F38" s="75"/>
+      <c r="G38" s="75"/>
+      <c r="H38" s="75"/>
+      <c r="I38" s="76"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B39" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="24"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="24"/>
+      <c r="I39" s="25"/>
+    </row>
+    <row r="40" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B40" s="20"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="21"/>
+      <c r="H40" s="21"/>
+      <c r="I40" s="22"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="21"/>
+      <c r="H41" s="21"/>
+      <c r="I41" s="22"/>
+    </row>
+    <row r="42" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B42" s="20"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="21"/>
+      <c r="H42" s="21"/>
+      <c r="I42" s="22"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="21"/>
+      <c r="H43" s="21"/>
+      <c r="I43" s="22"/>
+    </row>
+    <row r="44" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="20"/>
+      <c r="C44" s="21"/>
+      <c r="D44" s="21"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="21"/>
+      <c r="H44" s="21"/>
+      <c r="I44" s="22"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="21"/>
+      <c r="H45" s="21"/>
+      <c r="I45" s="22"/>
+    </row>
+    <row r="46" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="20"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="21"/>
+      <c r="H46" s="21"/>
+      <c r="I46" s="22"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="21"/>
+      <c r="H47" s="21"/>
+      <c r="I47" s="22"/>
+    </row>
+    <row r="48" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B48" s="20"/>
+      <c r="C48" s="21"/>
+      <c r="D48" s="21"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="21"/>
+      <c r="H48" s="21"/>
+      <c r="I48" s="22"/>
+    </row>
+    <row r="49" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B49" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="C49" s="21"/>
+      <c r="D49" s="21"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="21"/>
+      <c r="H49" s="21"/>
+      <c r="I49" s="22"/>
+    </row>
+    <row r="50" spans="2:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C50" s="21"/>
+      <c r="D50" s="21"/>
+      <c r="E50" s="21"/>
+      <c r="F50" s="21"/>
+      <c r="G50" s="21"/>
+      <c r="H50" s="21"/>
+      <c r="I50" s="22"/>
+    </row>
+    <row r="51" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B51" s="65" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="55"/>
-      <c r="D33" s="55"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="55"/>
-      <c r="H33" s="55"/>
-      <c r="I33" s="56"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="54" t="s">
-        <v>48</v>
-      </c>
-      <c r="C34" s="55"/>
-      <c r="D34" s="55"/>
-      <c r="E34" s="55"/>
-      <c r="F34" s="55"/>
-      <c r="G34" s="55"/>
-      <c r="H34" s="55"/>
-      <c r="I34" s="56"/>
-    </row>
-    <row r="35" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="54"/>
-      <c r="C35" s="55"/>
-      <c r="D35" s="55"/>
-      <c r="E35" s="55"/>
-      <c r="F35" s="55"/>
-      <c r="G35" s="55"/>
-      <c r="H35" s="55"/>
-      <c r="I35" s="56"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="54" t="s">
-        <v>9</v>
-      </c>
-      <c r="C36" s="55"/>
-      <c r="D36" s="55"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="55"/>
-      <c r="H36" s="55"/>
-      <c r="I36" s="56"/>
-    </row>
-    <row r="37" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="57"/>
-      <c r="C37" s="58"/>
-      <c r="D37" s="58"/>
-      <c r="E37" s="58"/>
-      <c r="F37" s="58"/>
-      <c r="G37" s="58"/>
-      <c r="H37" s="58"/>
-      <c r="I37" s="59"/>
-    </row>
-    <row r="38" spans="2:9" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="60" t="s">
-        <v>49</v>
-      </c>
-      <c r="C38" s="61"/>
-      <c r="D38" s="61"/>
-      <c r="E38" s="61"/>
-      <c r="F38" s="61"/>
-      <c r="G38" s="61"/>
-      <c r="H38" s="61"/>
-      <c r="I38" s="62"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="66" t="s">
-        <v>10</v>
-      </c>
-      <c r="C39" s="67"/>
-      <c r="D39" s="67"/>
-      <c r="E39" s="67"/>
-      <c r="F39" s="67"/>
-      <c r="G39" s="67"/>
-      <c r="H39" s="67"/>
-      <c r="I39" s="68"/>
-    </row>
-    <row r="40" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B40" s="54"/>
-      <c r="C40" s="55"/>
-      <c r="D40" s="55"/>
-      <c r="E40" s="55"/>
-      <c r="F40" s="55"/>
-      <c r="G40" s="55"/>
-      <c r="H40" s="55"/>
-      <c r="I40" s="56"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="54" t="s">
-        <v>11</v>
-      </c>
-      <c r="C41" s="55"/>
-      <c r="D41" s="55"/>
-      <c r="E41" s="55"/>
-      <c r="F41" s="55"/>
-      <c r="G41" s="55"/>
-      <c r="H41" s="55"/>
-      <c r="I41" s="56"/>
-    </row>
-    <row r="42" spans="2:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B42" s="54"/>
-      <c r="C42" s="55"/>
-      <c r="D42" s="55"/>
-      <c r="E42" s="55"/>
-      <c r="F42" s="55"/>
-      <c r="G42" s="55"/>
-      <c r="H42" s="55"/>
-      <c r="I42" s="56"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="54" t="s">
-        <v>50</v>
-      </c>
-      <c r="C43" s="55"/>
-      <c r="D43" s="55"/>
-      <c r="E43" s="55"/>
-      <c r="F43" s="55"/>
-      <c r="G43" s="55"/>
-      <c r="H43" s="55"/>
-      <c r="I43" s="56"/>
-    </row>
-    <row r="44" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B44" s="54"/>
-      <c r="C44" s="55"/>
-      <c r="D44" s="55"/>
-      <c r="E44" s="55"/>
-      <c r="F44" s="55"/>
-      <c r="G44" s="55"/>
-      <c r="H44" s="55"/>
-      <c r="I44" s="56"/>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B45" s="54" t="s">
+      <c r="C51" s="66"/>
+      <c r="D51" s="66"/>
+      <c r="E51" s="66"/>
+      <c r="F51" s="66"/>
+      <c r="G51" s="66"/>
+      <c r="H51" s="66"/>
+      <c r="I51" s="67"/>
+    </row>
+    <row r="52" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="26"/>
+      <c r="C52" s="27"/>
+      <c r="D52" s="27"/>
+      <c r="E52" s="27"/>
+      <c r="F52" s="27"/>
+      <c r="G52" s="27"/>
+      <c r="H52" s="27"/>
+      <c r="I52" s="28"/>
+    </row>
+    <row r="53" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="30" t="s">
+        <v>16</v>
+      </c>
+      <c r="C53" s="31"/>
+      <c r="D53" s="31"/>
+      <c r="E53" s="31"/>
+      <c r="F53" s="31"/>
+      <c r="G53" s="31"/>
+      <c r="H53" s="31"/>
+      <c r="I53" s="32"/>
+    </row>
+    <row r="54" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="29"/>
+      <c r="C54" s="16"/>
+      <c r="D54" s="16"/>
+      <c r="E54" s="16"/>
+      <c r="F54" s="16"/>
+      <c r="G54" s="16"/>
+      <c r="H54" s="16"/>
+      <c r="I54" s="17"/>
+    </row>
+    <row r="55" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="12"/>
+      <c r="C55" s="13"/>
+      <c r="D55" s="13"/>
+      <c r="E55" s="13"/>
+      <c r="F55" s="13"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="13"/>
+      <c r="I55" s="18"/>
+    </row>
+    <row r="56" spans="2:9" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="12"/>
+      <c r="C56" s="13"/>
+      <c r="D56" s="13"/>
+      <c r="E56" s="13"/>
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="13"/>
+      <c r="I56" s="18"/>
+    </row>
+    <row r="57" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="12"/>
+      <c r="C57" s="13"/>
+      <c r="D57" s="13"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="13"/>
+      <c r="I57" s="18"/>
+    </row>
+    <row r="58" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="12"/>
+      <c r="C58" s="13"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="13"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="13"/>
+      <c r="I58" s="18"/>
+    </row>
+    <row r="59" spans="2:9" ht="89.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="14"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
+      <c r="I59" s="19"/>
+    </row>
+    <row r="60" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="62" t="s">
         <v>51</v>
       </c>
-      <c r="C45" s="55"/>
-      <c r="D45" s="55"/>
-      <c r="E45" s="55"/>
-      <c r="F45" s="55"/>
-      <c r="G45" s="55"/>
-      <c r="H45" s="55"/>
-      <c r="I45" s="56"/>
-    </row>
-    <row r="46" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="54"/>
-      <c r="C46" s="55"/>
-      <c r="D46" s="55"/>
-      <c r="E46" s="55"/>
-      <c r="F46" s="55"/>
-      <c r="G46" s="55"/>
-      <c r="H46" s="55"/>
-      <c r="I46" s="56"/>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="54" t="s">
-        <v>12</v>
-      </c>
-      <c r="C47" s="55"/>
-      <c r="D47" s="55"/>
-      <c r="E47" s="55"/>
-      <c r="F47" s="55"/>
-      <c r="G47" s="55"/>
-      <c r="H47" s="55"/>
-      <c r="I47" s="56"/>
-    </row>
-    <row r="48" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="54"/>
-      <c r="C48" s="55"/>
-      <c r="D48" s="55"/>
-      <c r="E48" s="55"/>
-      <c r="F48" s="55"/>
-      <c r="G48" s="55"/>
-      <c r="H48" s="55"/>
-      <c r="I48" s="56"/>
-    </row>
-    <row r="49" spans="2:9" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B49" s="54" t="s">
-        <v>34</v>
-      </c>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="55"/>
-      <c r="F49" s="55"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="56"/>
-    </row>
-    <row r="50" spans="2:9" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="54" t="s">
-        <v>35</v>
-      </c>
-      <c r="C50" s="55"/>
-      <c r="D50" s="55"/>
-      <c r="E50" s="55"/>
-      <c r="F50" s="55"/>
-      <c r="G50" s="55"/>
-      <c r="H50" s="55"/>
-      <c r="I50" s="56"/>
-    </row>
-    <row r="51" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="89" t="s">
-        <v>30</v>
-      </c>
-      <c r="C51" s="90"/>
-      <c r="D51" s="90"/>
-      <c r="E51" s="90"/>
-      <c r="F51" s="90"/>
-      <c r="G51" s="90"/>
-      <c r="H51" s="90"/>
-      <c r="I51" s="91"/>
-    </row>
-    <row r="52" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="122"/>
-      <c r="C52" s="123"/>
-      <c r="D52" s="123"/>
-      <c r="E52" s="123"/>
-      <c r="F52" s="123"/>
-      <c r="G52" s="123"/>
-      <c r="H52" s="123"/>
-      <c r="I52" s="124"/>
-    </row>
-    <row r="53" spans="2:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B53" s="86" t="s">
-        <v>17</v>
-      </c>
-      <c r="C53" s="87"/>
-      <c r="D53" s="87"/>
-      <c r="E53" s="87"/>
-      <c r="F53" s="87"/>
-      <c r="G53" s="87"/>
-      <c r="H53" s="87"/>
-      <c r="I53" s="88"/>
-    </row>
-    <row r="54" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B54" s="114"/>
-      <c r="C54" s="115"/>
-      <c r="D54" s="115"/>
-      <c r="E54" s="115"/>
-      <c r="F54" s="115"/>
-      <c r="G54" s="115"/>
-      <c r="H54" s="115"/>
-      <c r="I54" s="116"/>
-    </row>
-    <row r="55" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B55" s="117"/>
-      <c r="C55" s="125"/>
-      <c r="D55" s="125"/>
-      <c r="E55" s="125"/>
-      <c r="F55" s="125"/>
-      <c r="G55" s="125"/>
-      <c r="H55" s="125"/>
-      <c r="I55" s="118"/>
-    </row>
-    <row r="56" spans="2:9" ht="88.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B56" s="117"/>
-      <c r="C56" s="125"/>
-      <c r="D56" s="125"/>
-      <c r="E56" s="125"/>
-      <c r="F56" s="125"/>
-      <c r="G56" s="125"/>
-      <c r="H56" s="125"/>
-      <c r="I56" s="118"/>
-    </row>
-    <row r="57" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B57" s="117"/>
-      <c r="C57" s="125"/>
-      <c r="D57" s="125"/>
-      <c r="E57" s="125"/>
-      <c r="F57" s="125"/>
-      <c r="G57" s="125"/>
-      <c r="H57" s="125"/>
-      <c r="I57" s="118"/>
-    </row>
-    <row r="58" spans="2:9" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B58" s="117"/>
-      <c r="C58" s="125"/>
-      <c r="D58" s="125"/>
-      <c r="E58" s="125"/>
-      <c r="F58" s="125"/>
-      <c r="G58" s="125"/>
-      <c r="H58" s="125"/>
-      <c r="I58" s="118"/>
-    </row>
-    <row r="59" spans="2:9" ht="89.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="119"/>
-      <c r="C59" s="120"/>
-      <c r="D59" s="120"/>
-      <c r="E59" s="120"/>
-      <c r="F59" s="120"/>
-      <c r="G59" s="120"/>
-      <c r="H59" s="120"/>
-      <c r="I59" s="121"/>
-    </row>
-    <row r="60" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="83" t="s">
+      <c r="C60" s="63"/>
+      <c r="D60" s="63"/>
+      <c r="E60" s="63"/>
+      <c r="F60" s="63"/>
+      <c r="G60" s="63"/>
+      <c r="H60" s="63"/>
+      <c r="I60" s="64"/>
+    </row>
+    <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B61" s="50" t="s">
+        <v>13</v>
+      </c>
+      <c r="C61" s="51"/>
+      <c r="D61" s="52" t="s">
+        <v>54</v>
+      </c>
+      <c r="E61" s="52"/>
+      <c r="F61" s="52"/>
+      <c r="G61" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="H61" s="55"/>
+      <c r="I61" s="56"/>
+    </row>
+    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B62" s="50" t="s">
+        <v>14</v>
+      </c>
+      <c r="C62" s="51"/>
+      <c r="D62" s="52" t="s">
+        <v>53</v>
+      </c>
+      <c r="E62" s="52"/>
+      <c r="F62" s="52"/>
+      <c r="G62" s="53"/>
+      <c r="H62" s="55"/>
+      <c r="I62" s="56"/>
+    </row>
+    <row r="63" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="50"/>
+      <c r="C63" s="51"/>
+      <c r="D63" s="52"/>
+      <c r="E63" s="52"/>
+      <c r="F63" s="52"/>
+      <c r="G63" s="53"/>
+      <c r="H63" s="55"/>
+      <c r="I63" s="56"/>
+    </row>
+    <row r="64" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B64" s="47" t="s">
         <v>52</v>
       </c>
-      <c r="C60" s="84"/>
-      <c r="D60" s="84"/>
-      <c r="E60" s="84"/>
-      <c r="F60" s="84"/>
-      <c r="G60" s="84"/>
-      <c r="H60" s="84"/>
-      <c r="I60" s="85"/>
-    </row>
-    <row r="61" spans="2:9" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B61" s="93" t="s">
+      <c r="C64" s="48"/>
+      <c r="D64" s="48"/>
+      <c r="E64" s="48"/>
+      <c r="F64" s="48"/>
+      <c r="G64" s="48"/>
+      <c r="H64" s="48"/>
+      <c r="I64" s="49"/>
+    </row>
+    <row r="65" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="50" t="s">
         <v>13</v>
       </c>
-      <c r="C61" s="94"/>
-      <c r="D61" s="92" t="s">
-        <v>16</v>
-      </c>
-      <c r="E61" s="92"/>
-      <c r="F61" s="92"/>
-      <c r="G61" s="95" t="s">
+      <c r="C65" s="51"/>
+      <c r="D65" s="52"/>
+      <c r="E65" s="52"/>
+      <c r="F65" s="52"/>
+      <c r="G65" s="53" t="s">
         <v>15</v>
       </c>
-      <c r="H61" s="82"/>
-      <c r="I61" s="28"/>
-    </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B62" s="93" t="s">
+      <c r="H65" s="55"/>
+      <c r="I65" s="56"/>
+    </row>
+    <row r="66" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B66" s="50" t="s">
         <v>14</v>
       </c>
-      <c r="C62" s="94"/>
-      <c r="D62" s="92" t="s">
-        <v>54</v>
-      </c>
-      <c r="E62" s="92"/>
-      <c r="F62" s="92"/>
-      <c r="G62" s="95"/>
-      <c r="H62" s="82"/>
-      <c r="I62" s="28"/>
-    </row>
-    <row r="63" spans="2:9" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="93"/>
-      <c r="C63" s="94"/>
-      <c r="D63" s="92"/>
-      <c r="E63" s="92"/>
-      <c r="F63" s="92"/>
-      <c r="G63" s="95"/>
-      <c r="H63" s="82"/>
-      <c r="I63" s="28"/>
-    </row>
-    <row r="64" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="96" t="s">
-        <v>53</v>
-      </c>
-      <c r="C64" s="97"/>
-      <c r="D64" s="97"/>
-      <c r="E64" s="97"/>
-      <c r="F64" s="97"/>
-      <c r="G64" s="97"/>
-      <c r="H64" s="97"/>
-      <c r="I64" s="98"/>
-    </row>
-    <row r="65" spans="2:9" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B65" s="93" t="s">
-        <v>13</v>
-      </c>
-      <c r="C65" s="94"/>
-      <c r="D65" s="92"/>
-      <c r="E65" s="92"/>
-      <c r="F65" s="92"/>
-      <c r="G65" s="95" t="s">
-        <v>15</v>
-      </c>
-      <c r="H65" s="82"/>
-      <c r="I65" s="28"/>
-    </row>
-    <row r="66" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B66" s="93" t="s">
-        <v>14</v>
-      </c>
-      <c r="C66" s="94"/>
-      <c r="D66" s="92"/>
-      <c r="E66" s="92"/>
-      <c r="F66" s="92"/>
-      <c r="G66" s="95"/>
-      <c r="H66" s="82"/>
-      <c r="I66" s="28"/>
+      <c r="C66" s="51"/>
+      <c r="D66" s="52"/>
+      <c r="E66" s="52"/>
+      <c r="F66" s="52"/>
+      <c r="G66" s="53"/>
+      <c r="H66" s="55"/>
+      <c r="I66" s="56"/>
     </row>
     <row r="67" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="101"/>
-      <c r="C67" s="102"/>
-      <c r="D67" s="103"/>
-      <c r="E67" s="103"/>
-      <c r="F67" s="103"/>
-      <c r="G67" s="99"/>
-      <c r="H67" s="100"/>
-      <c r="I67" s="30"/>
+      <c r="B67" s="59"/>
+      <c r="C67" s="60"/>
+      <c r="D67" s="61"/>
+      <c r="E67" s="61"/>
+      <c r="F67" s="61"/>
+      <c r="G67" s="54"/>
+      <c r="H67" s="57"/>
+      <c r="I67" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="81">
-    <mergeCell ref="B57:D59"/>
-    <mergeCell ref="E54:G56"/>
-    <mergeCell ref="E57:G59"/>
-    <mergeCell ref="H54:I56"/>
-    <mergeCell ref="H57:I59"/>
-    <mergeCell ref="B49:I49"/>
-    <mergeCell ref="B50:I50"/>
-    <mergeCell ref="B32:I32"/>
-    <mergeCell ref="B33:I33"/>
-    <mergeCell ref="B39:I40"/>
-    <mergeCell ref="B41:I42"/>
-    <mergeCell ref="B43:I44"/>
-    <mergeCell ref="B45:I46"/>
-    <mergeCell ref="B47:I48"/>
-    <mergeCell ref="B52:I52"/>
-    <mergeCell ref="B54:D56"/>
-    <mergeCell ref="B18:I18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="B22:E22"/>
-    <mergeCell ref="H20:I22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="B64:I64"/>
-    <mergeCell ref="B65:C65"/>
-    <mergeCell ref="D65:F65"/>
-    <mergeCell ref="G65:G67"/>
-    <mergeCell ref="H65:I67"/>
-    <mergeCell ref="B66:C67"/>
-    <mergeCell ref="D66:F67"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H10:H11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="B1:C5"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="D2:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B36:I37"/>
+    <mergeCell ref="B38:I38"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B7:I9"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B26:I26"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="B11:D11"/>
     <mergeCell ref="H61:I63"/>
     <mergeCell ref="B60:I60"/>
     <mergeCell ref="B53:I53"/>
@@ -2630,37 +2627,40 @@
     <mergeCell ref="B29:I29"/>
     <mergeCell ref="B30:I30"/>
     <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B36:I37"/>
-    <mergeCell ref="B38:I38"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B7:I9"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B26:I26"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="B1:C5"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="D2:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H10:H11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B65:C65"/>
+    <mergeCell ref="D65:F65"/>
+    <mergeCell ref="G65:G67"/>
+    <mergeCell ref="H65:I67"/>
+    <mergeCell ref="B66:C67"/>
+    <mergeCell ref="D66:F67"/>
+    <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B54:D56"/>
+    <mergeCell ref="B18:I18"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="H20:I22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B32:I32"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="B39:I40"/>
+    <mergeCell ref="B41:I42"/>
+    <mergeCell ref="B43:I44"/>
+    <mergeCell ref="B45:I46"/>
+    <mergeCell ref="B47:I48"/>
+    <mergeCell ref="B57:D59"/>
+    <mergeCell ref="E54:G56"/>
+    <mergeCell ref="E57:G59"/>
+    <mergeCell ref="H54:I56"/>
+    <mergeCell ref="H57:I59"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G14:G17" xr:uid="{C164E967-E733-492B-B646-A77CBB30BFA0}">
@@ -2680,15 +2680,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B823524E7585C14FA589DA6EA00187E3" ma:contentTypeVersion="17" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="50b97ae076214f52965bc923a1b0262e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="98b65742-7606-4aba-8ffb-70ac9bc50cd0" xmlns:ns3="30ba6132-0b50-445c-b091-6b36769966f5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="11b9c15a5bd2ebfec78f7ebeae66ec3d" ns2:_="" ns3:_="">
     <xsd:import namespace="98b65742-7606-4aba-8ffb-70ac9bc50cd0"/>
@@ -2937,6 +2928,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2949,14 +2949,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA83204B-C9C6-4F47-A347-B0DE6EF03566}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2975,6 +2967,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1ED24F7-12A7-4C45-A208-5E216D4E5BCE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{343F90F2-9DD9-41F8-A266-0D3FA1D7C8B8}">
   <ds:schemaRefs>

</xml_diff>